<commit_message>
test(SPARK-197): add owner approval API and UAT QA evidence
</commit_message>
<xml_diff>
--- a/docs/04-testing/test-cases/SmartParking_User_Master_TestCases.xlsx
+++ b/docs/04-testing/test-cases/SmartParking_User_Master_TestCases.xlsx
@@ -2,15 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R50ddd08f443840f8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Report" sheetId="2" r:id="R5396d8a80f24487e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Case List" sheetId="3" r:id="Rf9c1566d641e4a4d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Migration Queue" sheetId="4" r:id="R3bb1a8158e7c4531"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR9_Owner_E2E" sheetId="5" r:id="Receac518851a4761"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR9_Auth_UI" sheetId="6" r:id="R7fd116b3117e4ae7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SP177_Planned_QA" sheetId="7" r:id="R18955f9149a14d60"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historical_Run_Index" sheetId="8" r:id="R677e544d193647a4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open_Findings" sheetId="9" r:id="R984cb7fcc5844fb7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R691ab5e3746647c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Report" sheetId="2" r:id="R71c94b6b354a4b5a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Case List" sheetId="3" r:id="R4e5ac3f28db2401f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Migration Queue" sheetId="4" r:id="R62809c317b7d4291"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR9_Owner_E2E" sheetId="5" r:id="Rdd44017c8c3849bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR9_Auth_UI" sheetId="6" r:id="Rb589c158085b4526"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SP177_Planned_QA" sheetId="7" r:id="Rc3df73c7ab10453d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historical_Run_Index" sheetId="8" r:id="Rc7ff4bac39c84483"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open_Findings" sheetId="9" r:id="Rc089b02a0c454bb3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SP197_Admin_Approval" sheetId="10" r:id="R3012a4c60de841f0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -25,7 +26,7 @@
     <x:numFmt numFmtId="200" formatCode="0.0%"/>
     <x:numFmt numFmtId="201" formatCode="0%"/>
   </x:numFmts>
-  <x:fonts count="9">
+  <x:fonts count="17">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -77,8 +78,53 @@
       <x:color rgb="FF15384A"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="14"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF284B63"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF18455A"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF566474"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF087F5B"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFA56C17"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF1F475E"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF22475E"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="11">
+  <x:fills count="19">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -130,6 +176,46 @@
         <x:fgColor rgb="FFDDECF2"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF102B38"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF4F5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF186274"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAFBF0"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF3DC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE7F7F4"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE7EDF2"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF9E9"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -138,7 +224,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="57">
+  <x:cellXfs count="84">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -234,6 +320,65 @@
     <x:xf numFmtId="200" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="8" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="200" fontId="8" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="15" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="15" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="15" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="15" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="16" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -570,7 +715,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="G7" t="str">
-        <x:v>1.1 REVIEW</x:v>
+        <x:v>1.2 REVIEW</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -651,12 +796,1686 @@
     <x:row r="16">
       <x:c r="B16" t="str">
         <x:v>Chưa được Leader phê duyệt. Đối chiếu docs repo trước khi commit.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="30" customHeight="1">
+      <x:c r="B18" s="81" t="str">
+        <x:v>2026-10-29</x:v>
+      </x:c>
+      <x:c r="C18" s="81" t="str">
+        <x:v>1.2</x:v>
+      </x:c>
+      <x:c r="D18" s="81" t="str">
+        <x:v>Append SPARK197 API/UAT</x:v>
+      </x:c>
+      <x:c r="E18" s="81" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="F18" s="81" t="str">
+        <x:v>20 PASS + 9 UNTESTED on PR9 SHA; Newman 17/17 assertions. Existing nine sheets retained.</x:v>
+      </x:c>
+      <x:c r="G18" s="81" t="str">
+        <x:v>Jira SPARK-197 / 2026-10-29</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="B2:G2"/>
   </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="2" max="2" width="19" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="29" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="44" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="42" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="40" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="17" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="17" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="14" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="11" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="14" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="58" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="16" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="28" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="52" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="26" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="32" customHeight="1">
+      <x:c r="B1" s="59" t="str">
+        <x:v>SMARTPARKING  |  SPARK-197 ADMIN APPROVE OWNER - API + UAT</x:v>
+      </x:c>
+      <x:c r="C1" s="59"/>
+      <x:c r="D1" s="59"/>
+      <x:c r="E1" s="59"/>
+      <x:c r="F1" s="59"/>
+      <x:c r="G1" s="59"/>
+      <x:c r="H1" s="59"/>
+      <x:c r="I1" s="59"/>
+      <x:c r="J1" s="59"/>
+      <x:c r="K1" s="59"/>
+      <x:c r="L1" s="59"/>
+      <x:c r="M1" s="59"/>
+      <x:c r="N1" s="59"/>
+      <x:c r="O1" s="59"/>
+      <x:c r="P1" s="59"/>
+      <x:c r="Q1" s="59"/>
+    </x:row>
+    <x:row r="2" ht="22" customHeight="1">
+      <x:c r="B2" s="60" t="str">
+        <x:v>Testing Jira</x:v>
+      </x:c>
+      <x:c r="C2" t="str">
+        <x:v>SPARK-197</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="22" customHeight="1">
+      <x:c r="B3" s="60" t="str">
+        <x:v>Baseline SHA</x:v>
+      </x:c>
+      <x:c r="C3" t="str">
+        <x:v>9952091294a9603ee53863fca2b454e6a11eb666</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="22" customHeight="1">
+      <x:c r="B4" s="60" t="str">
+        <x:v>Scope</x:v>
+      </x:c>
+      <x:c r="C4" t="str">
+        <x:v>UserService · Admin Owner approval / rejection</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="23" customHeight="1">
+      <x:c r="B5" s="62" t="str">
+        <x:v>QA UAT PASS</x:v>
+      </x:c>
+      <x:c r="C5" s="62" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="D5" s="62" t="str">
+        <x:v>Newman/API PASS</x:v>
+      </x:c>
+      <x:c r="E5" s="62" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F5" s="62" t="str">
+        <x:v>Untested</x:v>
+      </x:c>
+      <x:c r="G5" s="62" t="n">
+        <x:v>9</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="23" customHeight="1">
+      <x:c r="B6" s="62" t="str">
+        <x:v>QA cases PASS</x:v>
+      </x:c>
+      <x:c r="C6" s="62" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="D6" s="62" t="str">
+        <x:v>FAIL</x:v>
+      </x:c>
+      <x:c r="E6" s="62" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F6" s="62" t="str">
+        <x:v>TOTAL CASES</x:v>
+      </x:c>
+      <x:c r="G6" s="62" t="n">
+        <x:v>29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="29" customHeight="1">
+      <x:c r="B7" s="64" t="str">
+        <x:v>Scope note: 10 manual UAT cases + 10 distinct Newman requests; direct API retests are corroboration, not double-counted. 9 gaps remain Untested.</x:v>
+      </x:c>
+      <x:c r="C7" s="64"/>
+      <x:c r="D7" s="64"/>
+      <x:c r="E7" s="64"/>
+      <x:c r="F7" s="64"/>
+      <x:c r="G7" s="64"/>
+      <x:c r="H7" s="64"/>
+      <x:c r="I7" s="64"/>
+      <x:c r="J7" s="64"/>
+      <x:c r="K7" s="64"/>
+      <x:c r="L7" s="64"/>
+      <x:c r="M7" s="64"/>
+      <x:c r="N7" s="64"/>
+      <x:c r="O7" s="64"/>
+      <x:c r="P7" s="64"/>
+      <x:c r="Q7" s="64"/>
+    </x:row>
+    <x:row r="8" ht="29" customHeight="1">
+      <x:c r="B8" s="64" t="str">
+        <x:v>All test data synthetic; no real identities or secrets. Result PASS applies only to executed cases, not to full Jira acceptance.</x:v>
+      </x:c>
+      <x:c r="C8" s="64"/>
+      <x:c r="D8" s="64"/>
+      <x:c r="E8" s="64"/>
+      <x:c r="F8" s="64"/>
+      <x:c r="G8" s="64"/>
+      <x:c r="H8" s="64"/>
+      <x:c r="I8" s="64"/>
+      <x:c r="J8" s="64"/>
+      <x:c r="K8" s="64"/>
+      <x:c r="L8" s="64"/>
+      <x:c r="M8" s="64"/>
+      <x:c r="N8" s="64"/>
+      <x:c r="O8" s="64"/>
+      <x:c r="P8" s="64"/>
+      <x:c r="Q8" s="64"/>
+    </x:row>
+    <x:row r="9" ht="34" customHeight="1">
+      <x:c r="B9" s="68" t="str">
+        <x:v>ID</x:v>
+      </x:c>
+      <x:c r="C9" s="68" t="str">
+        <x:v>Test Case Description</x:v>
+      </x:c>
+      <x:c r="D9" s="68" t="str">
+        <x:v>Test Case Procedure</x:v>
+      </x:c>
+      <x:c r="E9" s="68" t="str">
+        <x:v>Expected Results</x:v>
+      </x:c>
+      <x:c r="F9" s="68" t="str">
+        <x:v>Inter-test case Dependence</x:v>
+      </x:c>
+      <x:c r="G9" s="68" t="str">
+        <x:v>Result</x:v>
+      </x:c>
+      <x:c r="H9" s="68" t="str">
+        <x:v>Test date</x:v>
+      </x:c>
+      <x:c r="I9" s="68" t="str">
+        <x:v>Tester</x:v>
+      </x:c>
+      <x:c r="J9" s="68" t="str">
+        <x:v>Number of tests</x:v>
+      </x:c>
+      <x:c r="K9" s="68" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="L9" s="68" t="str">
+        <x:v>% Passed</x:v>
+      </x:c>
+      <x:c r="M9" s="68" t="str">
+        <x:v>Note / Actual</x:v>
+      </x:c>
+      <x:c r="N9" s="68" t="str">
+        <x:v>Testing Jira</x:v>
+      </x:c>
+      <x:c r="O9" s="68" t="str">
+        <x:v>Baseline commit</x:v>
+      </x:c>
+      <x:c r="P9" s="68" t="str">
+        <x:v>Evidence / source</x:v>
+      </x:c>
+      <x:c r="Q9" s="68" t="str">
+        <x:v>Scenario type</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="50" customHeight="1">
+      <x:c r="B10" s="26" t="str">
+        <x:v>[SP197-UAT-01]</x:v>
+      </x:c>
+      <x:c r="C10" s="26" t="str">
+        <x:v>Owner A business registration + lot setup</x:v>
+      </x:c>
+      <x:c r="D10" s="26" t="str">
+        <x:v>Sign Up &gt; Business; complete outdoor lot wizard; save lot setup</x:v>
+      </x:c>
+      <x:c r="E10" s="26" t="str">
+        <x:v>Valid QA Owner and lot submission are accepted</x:v>
+      </x:c>
+      <x:c r="F10" s="26" t="str">
+        <x:v>New QA email alias, QA services healthy</x:v>
+      </x:c>
+      <x:c r="G10" s="70" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H10" s="26" t="str">
+        <x:v>2026-10-29</x:v>
+      </x:c>
+      <x:c r="I10" s="26" t="str">
+        <x:v>QA Tester</x:v>
+      </x:c>
+      <x:c r="J10" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K10" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L10" s="51" t="n">
+        <x:f>IFERROR(K10/J10,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M10" s="26" t="str">
+        <x:v>Registered A; lot saved with 10 planned slots</x:v>
+      </x:c>
+      <x:c r="N10" s="26" t="str">
+        <x:v>SPARK-197</x:v>
+      </x:c>
+      <x:c r="O10" s="26" t="str">
+        <x:v>9952091294a9603ee53863fca2b454e6a11eb666</x:v>
+      </x:c>
+      <x:c r="P10" s="26" t="str">
+        <x:v>UAT screenshot: image(20261029-102348).png; user walkthrough</x:v>
+      </x:c>
+      <x:c r="Q10" s="26" t="str">
+        <x:v>UAT / onboarding</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="50" customHeight="1">
+      <x:c r="B11" s="26" t="str">
+        <x:v>[SP197-UAT-02]</x:v>
+      </x:c>
+      <x:c r="C11" s="26" t="str">
+        <x:v>Owner A email OTP + pending status</x:v>
+      </x:c>
+      <x:c r="D11" s="26" t="str">
+        <x:v>Retrieve real Gmail OTP and verify; inspect Admin Pending Review</x:v>
+      </x:c>
+      <x:c r="E11" s="26" t="str">
+        <x:v>Verified application moves to pending Admin review</x:v>
+      </x:c>
+      <x:c r="F11" s="26" t="str">
+        <x:v>Registered Owner A; inbox available</x:v>
+      </x:c>
+      <x:c r="G11" s="70" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H11" s="26" t="str">
+        <x:v>2026-10-29</x:v>
+      </x:c>
+      <x:c r="I11" s="26" t="str">
+        <x:v>QA Tester</x:v>
+      </x:c>
+      <x:c r="J11" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K11" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L11" s="51" t="n">
+        <x:f>IFERROR(K11/J11,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M11" s="26" t="str">
+        <x:v>Application Submitted; verified pending application visible to Admin</x:v>
+      </x:c>
+      <x:c r="N11" s="26" t="str">
+        <x:v>SPARK-197</x:v>
+      </x:c>
+      <x:c r="O11" s="26" t="str">
+        <x:v>9952091294a9603ee53863fca2b454e6a11eb666</x:v>
+      </x:c>
+      <x:c r="P11" s="26" t="str">
+        <x:v>UAT: image(20261029-102502).png; Admin pending screenshot</x:v>
+      </x:c>
+      <x:c r="Q11" s="26" t="str">
+        <x:v>UAT / eligibility</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="50" customHeight="1">
+      <x:c r="B12" s="26" t="str">
+        <x:v>[SP197-UAT-03]</x:v>
+      </x:c>
+      <x:c r="C12" s="26" t="str">
+        <x:v>Pending Owner cannot access dashboard</x:v>
+      </x:c>
+      <x:c r="D12" s="26" t="str">
+        <x:v>Sign in as Owner A before Admin approval</x:v>
+      </x:c>
+      <x:c r="E12" s="26" t="str">
+        <x:v>Pending account does not reach Owner dashboard</x:v>
+      </x:c>
+      <x:c r="F12" s="26" t="str">
+        <x:v>Owner A pending and verified</x:v>
+      </x:c>
+      <x:c r="G12" s="70" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H12" s="26" t="str">
+        <x:v>2026-10-29</x:v>
+      </x:c>
+      <x:c r="I12" s="26" t="str">
+        <x:v>QA Tester</x:v>
+      </x:c>
+      <x:c r="J12" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K12" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L12" s="51" t="n">
+        <x:f>IFERROR(K12/J12,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M12" s="26" t="str">
+        <x:v>Sign-in returned Application Submitted (not dashboard); backend control not separately inspected</x:v>
+      </x:c>
+      <x:c r="N12" s="26" t="str">
+        <x:v>SPARK-197</x:v>
+      </x:c>
+      <x:c r="O12" s="26" t="str">
+        <x:v>9952091294a9603ee53863fca2b454e6a11eb666</x:v>
+      </x:c>
+      <x:c r="P12" s="26" t="str">
+        <x:v>UAT user-confirmed sign-in; image(20261029-102844).png</x:v>
+      </x:c>
+      <x:c r="Q12" s="26" t="str">
+        <x:v>UAT / access control</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="50" customHeight="1">
+      <x:c r="B13" s="26" t="str">
+        <x:v>[SP197-UAT-04]</x:v>
+      </x:c>
+      <x:c r="C13" s="26" t="str">
+        <x:v>Admin application review details</x:v>
+      </x:c>
+      <x:c r="D13" s="26" t="str">
+        <x:v>Admin view pending applications; expand lot setup</x:v>
+      </x:c>
+      <x:c r="E13" s="26" t="str">
+        <x:v>Business details, contact verification, setup/rates visible</x:v>
+      </x:c>
+      <x:c r="F13" s="26" t="str">
+        <x:v>Admin session; Owner A/B pending at relevant time</x:v>
+      </x:c>
+      <x:c r="G13" s="70" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H13" s="26" t="str">
+        <x:v>2026-10-29</x:v>
+      </x:c>
+      <x:c r="I13" s="26" t="str">
+        <x:v>QA Tester</x:v>
+      </x:c>
+      <x:c r="J13" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K13" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L13" s="51" t="n">
+        <x:f>IFERROR(K13/J13,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M13" s="26" t="str">
+        <x:v>Admin listed requests and showed lot setup and rates</x:v>
+      </x:c>
+      <x:c r="N13" s="26" t="str">
+        <x:v>SPARK-197</x:v>
+      </x:c>
+      <x:c r="O13" s="26" t="str">
+        <x:v>9952091294a9603ee53863fca2b454e6a11eb666</x:v>
+      </x:c>
+      <x:c r="P13" s="26" t="str">
+        <x:v>UAT: image(20261029-105428).png (Owner B)</x:v>
+      </x:c>
+      <x:c r="Q13" s="26" t="str">
+        <x:v>UAT / admin detail</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="50" customHeight="1">
+      <x:c r="B14" s="26" t="str">
+        <x:v>[SP197-UAT-05]</x:v>
+      </x:c>
+      <x:c r="C14" s="26" t="str">
+        <x:v>Admin approves Owner A with review note</x:v>
+      </x:c>
+      <x:c r="D14" s="26" t="str">
+        <x:v>Admin Approve only SPARK197 QA Parking A; refresh</x:v>
+      </x:c>
+      <x:c r="E14" s="26" t="str">
+        <x:v>Application approved; review note persisted; pending item removed</x:v>
+      </x:c>
+      <x:c r="F14" s="26" t="str">
+        <x:v>Verified eligible Owner A pending</x:v>
+      </x:c>
+      <x:c r="G14" s="70" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H14" s="26" t="str">
+        <x:v>2026-10-29</x:v>
+      </x:c>
+      <x:c r="I14" s="26" t="str">
+        <x:v>QA Tester</x:v>
+      </x:c>
+      <x:c r="J14" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K14" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L14" s="51" t="n">
+        <x:f>IFERROR(K14/J14,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M14" s="26" t="str">
+        <x:v>APPROVED, Previously Reviewed; review note shown</x:v>
+      </x:c>
+      <x:c r="N14" s="26" t="str">
+        <x:v>SPARK-197</x:v>
+      </x:c>
+      <x:c r="O14" s="26" t="str">
+        <x:v>9952091294a9603ee53863fca2b454e6a11eb666</x:v>
+      </x:c>
+      <x:c r="P14" s="26" t="str">
+        <x:v>EV-UAT-01: SP197_Admin_Final_Decisions.png; original image(20261029-103346).png</x:v>
+      </x:c>
+      <x:c r="Q14" s="26" t="str">
+        <x:v>UAT / approve</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="50" customHeight="1">
+      <x:c r="B15" s="26" t="str">
+        <x:v>[SP197-UAT-06]</x:v>
+      </x:c>
+      <x:c r="C15" s="26" t="str">
+        <x:v>Approved Owner access + site activation</x:v>
+      </x:c>
+      <x:c r="D15" s="26" t="str">
+        <x:v>Sign in as Owner A; inspect Owner Overview, Site &amp; Staff</x:v>
+      </x:c>
+      <x:c r="E15" s="26" t="str">
+        <x:v>Approved Owner accesses dashboard and has active site</x:v>
+      </x:c>
+      <x:c r="F15" s="26" t="str">
+        <x:v>Admin approval persisted</x:v>
+      </x:c>
+      <x:c r="G15" s="70" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H15" s="26" t="str">
+        <x:v>2026-10-29</x:v>
+      </x:c>
+      <x:c r="I15" s="26" t="str">
+        <x:v>QA Tester</x:v>
+      </x:c>
+      <x:c r="J15" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K15" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L15" s="51" t="n">
+        <x:f>IFERROR(K15/J15,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M15" s="26" t="str">
+        <x:v>Owner Overview accessible; 1 site ACTIVE; physical slots 0</x:v>
+      </x:c>
+      <x:c r="N15" s="26" t="str">
+        <x:v>SPARK-197</x:v>
+      </x:c>
+      <x:c r="O15" s="26" t="str">
+        <x:v>9952091294a9603ee53863fca2b454e6a11eb666</x:v>
+      </x:c>
+      <x:c r="P15" s="26" t="str">
+        <x:v>EV-UAT-04: SP197_Owner_Approved_Dashboard.png; originals image(20261029-103429).png, image(20261029-103529).png</x:v>
+      </x:c>
+      <x:c r="Q15" s="26" t="str">
+        <x:v>UAT / cross-service</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="50" customHeight="1">
+      <x:c r="B16" s="26" t="str">
+        <x:v>[SP197-UAT-07]</x:v>
+      </x:c>
+      <x:c r="C16" s="26" t="str">
+        <x:v>Admin rejects Owner B with review note</x:v>
+      </x:c>
+      <x:c r="D16" s="26" t="str">
+        <x:v>Create and verify Owner B; Admin select Reject with QA review note</x:v>
+      </x:c>
+      <x:c r="E16" s="26" t="str">
+        <x:v>Application rejected; reason retained; Owner A remains approved</x:v>
+      </x:c>
+      <x:c r="F16" s="26" t="str">
+        <x:v>Verified QA Owner B pending</x:v>
+      </x:c>
+      <x:c r="G16" s="70" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H16" s="26" t="str">
+        <x:v>2026-10-29</x:v>
+      </x:c>
+      <x:c r="I16" s="26" t="str">
+        <x:v>QA Tester</x:v>
+      </x:c>
+      <x:c r="J16" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K16" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L16" s="51" t="n">
+        <x:f>IFERROR(K16/J16,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M16" s="26" t="str">
+        <x:v>REJECTED listed Previously Reviewed; QA review note retained; A still APPROVED</x:v>
+      </x:c>
+      <x:c r="N16" s="26" t="str">
+        <x:v>SPARK-197</x:v>
+      </x:c>
+      <x:c r="O16" s="26" t="str">
+        <x:v>9952091294a9603ee53863fca2b454e6a11eb666</x:v>
+      </x:c>
+      <x:c r="P16" s="26" t="str">
+        <x:v>EV-UAT-01: SP197_Admin_Final_Decisions.png; original image(20261029-105436).png</x:v>
+      </x:c>
+      <x:c r="Q16" s="26" t="str">
+        <x:v>UAT / reject</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="50" customHeight="1">
+      <x:c r="B17" s="26" t="str">
+        <x:v>[SP197-UAT-08]</x:v>
+      </x:c>
+      <x:c r="C17" s="26" t="str">
+        <x:v>Rejected Owner cannot log in</x:v>
+      </x:c>
+      <x:c r="D17" s="26" t="str">
+        <x:v>After rejecting Owner B, attempt password sign in</x:v>
+      </x:c>
+      <x:c r="E17" s="26" t="str">
+        <x:v>No Owner dashboard; explicit rejected-application error</x:v>
+      </x:c>
+      <x:c r="F17" s="26" t="str">
+        <x:v>Owner B REJECTED</x:v>
+      </x:c>
+      <x:c r="G17" s="70" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H17" s="26" t="str">
+        <x:v>2026-10-29</x:v>
+      </x:c>
+      <x:c r="I17" s="26" t="str">
+        <x:v>QA Tester</x:v>
+      </x:c>
+      <x:c r="J17" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K17" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L17" s="51" t="n">
+        <x:f>IFERROR(K17/J17,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M17" s="26" t="str">
+        <x:v>Error: Your account application was rejected. Please contact the administrator.</x:v>
+      </x:c>
+      <x:c r="N17" s="26" t="str">
+        <x:v>SPARK-197</x:v>
+      </x:c>
+      <x:c r="O17" s="26" t="str">
+        <x:v>9952091294a9603ee53863fca2b454e6a11eb666</x:v>
+      </x:c>
+      <x:c r="P17" s="26" t="str">
+        <x:v>EV-UAT-02: SP197_Rejected_Login.png; original image(20261029-105544).png</x:v>
+      </x:c>
+      <x:c r="Q17" s="26" t="str">
+        <x:v>UAT / access control</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="50" customHeight="1">
+      <x:c r="B18" s="26" t="str">
+        <x:v>[SP197-UAT-09]</x:v>
+      </x:c>
+      <x:c r="C18" s="26" t="str">
+        <x:v>Approval email delivered to real inbox</x:v>
+      </x:c>
+      <x:c r="D18" s="26" t="str">
+        <x:v>Inspect test mailbox for Owner A decision</x:v>
+      </x:c>
+      <x:c r="E18" s="26" t="str">
+        <x:v>Approved decision email is received</x:v>
+      </x:c>
+      <x:c r="F18" s="26" t="str">
+        <x:v>Owner A approved; mail delivery worker active</x:v>
+      </x:c>
+      <x:c r="G18" s="70" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H18" s="26" t="str">
+        <x:v>2026-10-29</x:v>
+      </x:c>
+      <x:c r="I18" s="26" t="str">
+        <x:v>QA Tester</x:v>
+      </x:c>
+      <x:c r="J18" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K18" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L18" s="51" t="n">
+        <x:f>IFERROR(K18/J18,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M18" s="26" t="str">
+        <x:v>Gmail: Your application is approved.; Admin notification sent</x:v>
+      </x:c>
+      <x:c r="N18" s="26" t="str">
+        <x:v>SPARK-197</x:v>
+      </x:c>
+      <x:c r="O18" s="26" t="str">
+        <x:v>9952091294a9603ee53863fca2b454e6a11eb666</x:v>
+      </x:c>
+      <x:c r="P18" s="26" t="str">
+        <x:v>EV-UAT-03: SP197_Approval_Rejection_Emails_Redacted.png; original image(20261029-105620).png</x:v>
+      </x:c>
+      <x:c r="Q18" s="26" t="str">
+        <x:v>UAT / notification</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="50" customHeight="1">
+      <x:c r="B19" s="26" t="str">
+        <x:v>[SP197-UAT-10]</x:v>
+      </x:c>
+      <x:c r="C19" s="26" t="str">
+        <x:v>Rejection email delivered to real inbox</x:v>
+      </x:c>
+      <x:c r="D19" s="26" t="str">
+        <x:v>Inspect test mailbox for Owner B decision</x:v>
+      </x:c>
+      <x:c r="E19" s="26" t="str">
+        <x:v>Rejected decision email is received</x:v>
+      </x:c>
+      <x:c r="F19" s="26" t="str">
+        <x:v>Owner B rejected; mail delivery worker active</x:v>
+      </x:c>
+      <x:c r="G19" s="70" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H19" s="26" t="str">
+        <x:v>2026-10-29</x:v>
+      </x:c>
+      <x:c r="I19" s="26" t="str">
+        <x:v>QA Tester</x:v>
+      </x:c>
+      <x:c r="J19" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K19" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L19" s="51" t="n">
+        <x:f>IFERROR(K19/J19,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M19" s="26" t="str">
+        <x:v>Gmail: Your application is rejected.; Admin notification sent</x:v>
+      </x:c>
+      <x:c r="N19" s="26" t="str">
+        <x:v>SPARK-197</x:v>
+      </x:c>
+      <x:c r="O19" s="26" t="str">
+        <x:v>9952091294a9603ee53863fca2b454e6a11eb666</x:v>
+      </x:c>
+      <x:c r="P19" s="26" t="str">
+        <x:v>EV-UAT-03: SP197_Approval_Rejection_Emails_Redacted.png; original image(20261029-105620).png</x:v>
+      </x:c>
+      <x:c r="Q19" s="26" t="str">
+        <x:v>UAT / notification</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="50" customHeight="1">
+      <x:c r="B20" s="26" t="str">
+        <x:v>[SP197-API-01]</x:v>
+      </x:c>
+      <x:c r="C20" s="26" t="str">
+        <x:v>Anonymous GET applications list</x:v>
+      </x:c>
+      <x:c r="D20" s="26" t="str">
+        <x:v>Without bearer JWT, GET /api/owner-applications</x:v>
+      </x:c>
+      <x:c r="E20" s="26" t="str">
+        <x:v>HTTP 401, no application data</x:v>
+      </x:c>
+      <x:c r="F20" s="26" t="str">
+        <x:v>QA UserService running</x:v>
+      </x:c>
+      <x:c r="G20" s="70" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H20" s="26" t="str">
+        <x:v>2026-10-29</x:v>
+      </x:c>
+      <x:c r="I20" s="26" t="str">
+        <x:v>QA Tester</x:v>
+      </x:c>
+      <x:c r="J20" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K20" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L20" s="51" t="n">
+        <x:f>IFERROR(K20/J20,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M20" s="26" t="str">
+        <x:v>Newman: HTTP 401; 1 assertion(s) PASS</x:v>
+      </x:c>
+      <x:c r="N20" s="26" t="str">
+        <x:v>SPARK-197</x:v>
+      </x:c>
+      <x:c r="O20" s="26" t="str">
+        <x:v>9952091294a9603ee53863fca2b454e6a11eb666</x:v>
+      </x:c>
+      <x:c r="P20" s="26" t="str">
+        <x:v>SPARK-197-Newman-Sanitized-Result.json; Anonymous list</x:v>
+      </x:c>
+      <x:c r="Q20" s="26" t="str">
+        <x:v>AUTH / no token</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="50" customHeight="1">
+      <x:c r="B21" s="26" t="str">
+        <x:v>[SP197-API-02]</x:v>
+      </x:c>
+      <x:c r="C21" s="26" t="str">
+        <x:v>Anonymous GET application detail</x:v>
+      </x:c>
+      <x:c r="D21" s="26" t="str">
+        <x:v>Without JWT, GET /api/owner-applications/{zero-guid}</x:v>
+      </x:c>
+      <x:c r="E21" s="26" t="str">
+        <x:v>HTTP 401</x:v>
+      </x:c>
+      <x:c r="F21" s="26" t="str">
+        <x:v>QA UserService running</x:v>
+      </x:c>
+      <x:c r="G21" s="70" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H21" s="26" t="str">
+        <x:v>2026-10-29</x:v>
+      </x:c>
+      <x:c r="I21" s="26" t="str">
+        <x:v>QA Tester</x:v>
+      </x:c>
+      <x:c r="J21" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K21" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L21" s="51" t="n">
+        <x:f>IFERROR(K21/J21,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M21" s="26" t="str">
+        <x:v>Newman: HTTP 401; 1 assertion(s) PASS</x:v>
+      </x:c>
+      <x:c r="N21" s="26" t="str">
+        <x:v>SPARK-197</x:v>
+      </x:c>
+      <x:c r="O21" s="26" t="str">
+        <x:v>9952091294a9603ee53863fca2b454e6a11eb666</x:v>
+      </x:c>
+      <x:c r="P21" s="26" t="str">
+        <x:v>SPARK-197-Newman-Sanitized-Result.json; Anonymous detail</x:v>
+      </x:c>
+      <x:c r="Q21" s="26" t="str">
+        <x:v>AUTH / no token</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="50" customHeight="1">
+      <x:c r="B22" s="26" t="str">
+        <x:v>[SP197-API-03]</x:v>
+      </x:c>
+      <x:c r="C22" s="26" t="str">
+        <x:v>Anonymous PATCH decision blocked</x:v>
+      </x:c>
+      <x:c r="D22" s="26" t="str">
+        <x:v>Without JWT, PATCH /api/owner-applications/{zero-guid}/review</x:v>
+      </x:c>
+      <x:c r="E22" s="26" t="str">
+        <x:v>HTTP 401; no review</x:v>
+      </x:c>
+      <x:c r="F22" s="26" t="str">
+        <x:v>QA UserService running</x:v>
+      </x:c>
+      <x:c r="G22" s="70" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H22" s="26" t="str">
+        <x:v>2026-10-29</x:v>
+      </x:c>
+      <x:c r="I22" s="26" t="str">
+        <x:v>QA Tester</x:v>
+      </x:c>
+      <x:c r="J22" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K22" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L22" s="51" t="n">
+        <x:f>IFERROR(K22/J22,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M22" s="26" t="str">
+        <x:v>Newman: HTTP 401; 1 assertion(s) PASS</x:v>
+      </x:c>
+      <x:c r="N22" s="26" t="str">
+        <x:v>SPARK-197</x:v>
+      </x:c>
+      <x:c r="O22" s="26" t="str">
+        <x:v>9952091294a9603ee53863fca2b454e6a11eb666</x:v>
+      </x:c>
+      <x:c r="P22" s="26" t="str">
+        <x:v>SPARK-197-Newman-Sanitized-Result.json; Anonymous review denied</x:v>
+      </x:c>
+      <x:c r="Q22" s="26" t="str">
+        <x:v>AUTH / no token</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="50" customHeight="1">
+      <x:c r="B23" s="26" t="str">
+        <x:v>[SP197-API-04]</x:v>
+      </x:c>
+      <x:c r="C23" s="26" t="str">
+        <x:v>Owner GET applications list denied</x:v>
+      </x:c>
+      <x:c r="D23" s="26" t="str">
+        <x:v>Owner A valid token; GET /api/owner-applications</x:v>
+      </x:c>
+      <x:c r="E23" s="26" t="str">
+        <x:v>HTTP 403</x:v>
+      </x:c>
+      <x:c r="F23" s="26" t="str">
+        <x:v>Owner A approved; valid Owner JWT</x:v>
+      </x:c>
+      <x:c r="G23" s="70" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H23" s="26" t="str">
+        <x:v>2026-10-29</x:v>
+      </x:c>
+      <x:c r="I23" s="26" t="str">
+        <x:v>QA Tester</x:v>
+      </x:c>
+      <x:c r="J23" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K23" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L23" s="51" t="n">
+        <x:f>IFERROR(K23/J23,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M23" s="26" t="str">
+        <x:v>Newman: HTTP 403; 1 assertion(s) PASS</x:v>
+      </x:c>
+      <x:c r="N23" s="26" t="str">
+        <x:v>SPARK-197</x:v>
+      </x:c>
+      <x:c r="O23" s="26" t="str">
+        <x:v>9952091294a9603ee53863fca2b454e6a11eb666</x:v>
+      </x:c>
+      <x:c r="P23" s="26" t="str">
+        <x:v>SPARK-197-Newman-Sanitized-Result.json; Owner list denied</x:v>
+      </x:c>
+      <x:c r="Q23" s="26" t="str">
+        <x:v>AUTH / owner scope</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="50" customHeight="1">
+      <x:c r="B24" s="26" t="str">
+        <x:v>[SP197-API-05]</x:v>
+      </x:c>
+      <x:c r="C24" s="26" t="str">
+        <x:v>Owner GET detail denied</x:v>
+      </x:c>
+      <x:c r="D24" s="26" t="str">
+        <x:v>Owner A valid token; GET /api/owner-applications/{zero-guid}</x:v>
+      </x:c>
+      <x:c r="E24" s="26" t="str">
+        <x:v>HTTP 403</x:v>
+      </x:c>
+      <x:c r="F24" s="26" t="str">
+        <x:v>Owner A approved; valid Owner JWT</x:v>
+      </x:c>
+      <x:c r="G24" s="70" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H24" s="26" t="str">
+        <x:v>2026-10-29</x:v>
+      </x:c>
+      <x:c r="I24" s="26" t="str">
+        <x:v>QA Tester</x:v>
+      </x:c>
+      <x:c r="J24" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K24" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L24" s="51" t="n">
+        <x:f>IFERROR(K24/J24,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M24" s="26" t="str">
+        <x:v>Newman: HTTP 403; 1 assertion(s) PASS</x:v>
+      </x:c>
+      <x:c r="N24" s="26" t="str">
+        <x:v>SPARK-197</x:v>
+      </x:c>
+      <x:c r="O24" s="26" t="str">
+        <x:v>9952091294a9603ee53863fca2b454e6a11eb666</x:v>
+      </x:c>
+      <x:c r="P24" s="26" t="str">
+        <x:v>SPARK-197-Newman-Sanitized-Result.json; Owner detail denied</x:v>
+      </x:c>
+      <x:c r="Q24" s="26" t="str">
+        <x:v>AUTH / owner scope</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="50" customHeight="1">
+      <x:c r="B25" s="26" t="str">
+        <x:v>[SP197-API-06]</x:v>
+      </x:c>
+      <x:c r="C25" s="26" t="str">
+        <x:v>Owner PATCH decision denied</x:v>
+      </x:c>
+      <x:c r="D25" s="26" t="str">
+        <x:v>Owner A valid token; PATCH /api/owner-applications/{zero-guid}/review</x:v>
+      </x:c>
+      <x:c r="E25" s="26" t="str">
+        <x:v>HTTP 403; no review</x:v>
+      </x:c>
+      <x:c r="F25" s="26" t="str">
+        <x:v>Owner A approved; valid Owner JWT</x:v>
+      </x:c>
+      <x:c r="G25" s="70" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H25" s="26" t="str">
+        <x:v>2026-10-29</x:v>
+      </x:c>
+      <x:c r="I25" s="26" t="str">
+        <x:v>QA Tester</x:v>
+      </x:c>
+      <x:c r="J25" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K25" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L25" s="51" t="n">
+        <x:f>IFERROR(K25/J25,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M25" s="26" t="str">
+        <x:v>Newman: HTTP 403; 1 assertion(s) PASS</x:v>
+      </x:c>
+      <x:c r="N25" s="26" t="str">
+        <x:v>SPARK-197</x:v>
+      </x:c>
+      <x:c r="O25" s="26" t="str">
+        <x:v>9952091294a9603ee53863fca2b454e6a11eb666</x:v>
+      </x:c>
+      <x:c r="P25" s="26" t="str">
+        <x:v>SPARK-197-Newman-Sanitized-Result.json; Owner review denied</x:v>
+      </x:c>
+      <x:c r="Q25" s="26" t="str">
+        <x:v>AUTH / owner scope</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="50" customHeight="1">
+      <x:c r="B26" s="26" t="str">
+        <x:v>[SP197-API-07]</x:v>
+      </x:c>
+      <x:c r="C26" s="26" t="str">
+        <x:v>Admin lists applications</x:v>
+      </x:c>
+      <x:c r="D26" s="26" t="str">
+        <x:v>Admin valid token; GET /api/owner-applications</x:v>
+      </x:c>
+      <x:c r="E26" s="26" t="str">
+        <x:v>HTTP 200; QA A approved and B rejected</x:v>
+      </x:c>
+      <x:c r="F26" s="26" t="str">
+        <x:v>Admin active; existing QA applications</x:v>
+      </x:c>
+      <x:c r="G26" s="70" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H26" s="26" t="str">
+        <x:v>2026-10-29</x:v>
+      </x:c>
+      <x:c r="I26" s="26" t="str">
+        <x:v>QA Tester</x:v>
+      </x:c>
+      <x:c r="J26" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K26" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L26" s="51" t="n">
+        <x:f>IFERROR(K26/J26,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M26" s="26" t="str">
+        <x:v>Newman: HTTP 200; 2 assertion(s) PASS; A approved / B rejected in list</x:v>
+      </x:c>
+      <x:c r="N26" s="26" t="str">
+        <x:v>SPARK-197</x:v>
+      </x:c>
+      <x:c r="O26" s="26" t="str">
+        <x:v>9952091294a9603ee53863fca2b454e6a11eb666</x:v>
+      </x:c>
+      <x:c r="P26" s="26" t="str">
+        <x:v>SPARK-197-Newman-Sanitized-Result.json; Admin list</x:v>
+      </x:c>
+      <x:c r="Q26" s="26" t="str">
+        <x:v>API / admin list</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="50" customHeight="1">
+      <x:c r="B27" s="26" t="str">
+        <x:v>[SP197-API-08]</x:v>
+      </x:c>
+      <x:c r="C27" s="26" t="str">
+        <x:v>Admin reads Approved Owner A</x:v>
+      </x:c>
+      <x:c r="D27" s="26" t="str">
+        <x:v>Admin valid token; GET detail with A ID read from list</x:v>
+      </x:c>
+      <x:c r="E27" s="26" t="str">
+        <x:v>HTTP 200; approved; reviewer/time and sent status present</x:v>
+      </x:c>
+      <x:c r="F27" s="26" t="str">
+        <x:v>Admin active; A approved</x:v>
+      </x:c>
+      <x:c r="G27" s="70" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H27" s="26" t="str">
+        <x:v>2026-10-29</x:v>
+      </x:c>
+      <x:c r="I27" s="26" t="str">
+        <x:v>QA Tester</x:v>
+      </x:c>
+      <x:c r="J27" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K27" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L27" s="51" t="n">
+        <x:f>IFERROR(K27/J27,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M27" s="26" t="str">
+        <x:v>Newman: HTTP 200; 4 assertion(s) PASS; reviewedBy/reviewedAt present, deliveryStatus sent</x:v>
+      </x:c>
+      <x:c r="N27" s="26" t="str">
+        <x:v>SPARK-197</x:v>
+      </x:c>
+      <x:c r="O27" s="26" t="str">
+        <x:v>9952091294a9603ee53863fca2b454e6a11eb666</x:v>
+      </x:c>
+      <x:c r="P27" s="26" t="str">
+        <x:v>SPARK-197-Newman-Sanitized-Result.json; Admin detail A</x:v>
+      </x:c>
+      <x:c r="Q27" s="26" t="str">
+        <x:v>API / detail audit</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="50" customHeight="1">
+      <x:c r="B28" s="26" t="str">
+        <x:v>[SP197-API-09]</x:v>
+      </x:c>
+      <x:c r="C28" s="26" t="str">
+        <x:v>Admin reads Rejected Owner B</x:v>
+      </x:c>
+      <x:c r="D28" s="26" t="str">
+        <x:v>Admin valid token; GET detail with B ID read from list</x:v>
+      </x:c>
+      <x:c r="E28" s="26" t="str">
+        <x:v>HTTP 200; rejected; reviewer/time and sent status present</x:v>
+      </x:c>
+      <x:c r="F28" s="26" t="str">
+        <x:v>Admin active; B rejected</x:v>
+      </x:c>
+      <x:c r="G28" s="70" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H28" s="26" t="str">
+        <x:v>2026-10-29</x:v>
+      </x:c>
+      <x:c r="I28" s="26" t="str">
+        <x:v>QA Tester</x:v>
+      </x:c>
+      <x:c r="J28" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K28" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L28" s="51" t="n">
+        <x:f>IFERROR(K28/J28,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M28" s="26" t="str">
+        <x:v>Newman: HTTP 200; 4 assertion(s) PASS; reviewedBy/reviewedAt present, deliveryStatus sent</x:v>
+      </x:c>
+      <x:c r="N28" s="26" t="str">
+        <x:v>SPARK-197</x:v>
+      </x:c>
+      <x:c r="O28" s="26" t="str">
+        <x:v>9952091294a9603ee53863fca2b454e6a11eb666</x:v>
+      </x:c>
+      <x:c r="P28" s="26" t="str">
+        <x:v>SPARK-197-Newman-Sanitized-Result.json; Admin detail B</x:v>
+      </x:c>
+      <x:c r="Q28" s="26" t="str">
+        <x:v>API / detail audit</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="50" customHeight="1">
+      <x:c r="B29" s="26" t="str">
+        <x:v>[SP197-API-10]</x:v>
+      </x:c>
+      <x:c r="C29" s="26" t="str">
+        <x:v>Admin GET nonexistent ID</x:v>
+      </x:c>
+      <x:c r="D29" s="26" t="str">
+        <x:v>Admin valid token; GET /api/owner-applications/{zero-guid}</x:v>
+      </x:c>
+      <x:c r="E29" s="26" t="str">
+        <x:v>HTTP 404; no record</x:v>
+      </x:c>
+      <x:c r="F29" s="26" t="str">
+        <x:v>Admin active; zero GUID non-existent</x:v>
+      </x:c>
+      <x:c r="G29" s="70" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H29" s="26" t="str">
+        <x:v>2026-10-29</x:v>
+      </x:c>
+      <x:c r="I29" s="26" t="str">
+        <x:v>QA Tester</x:v>
+      </x:c>
+      <x:c r="J29" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K29" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L29" s="51" t="n">
+        <x:f>IFERROR(K29/J29,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M29" s="26" t="str">
+        <x:v>Newman: HTTP 404; 1 assertion(s) PASS</x:v>
+      </x:c>
+      <x:c r="N29" s="26" t="str">
+        <x:v>SPARK-197</x:v>
+      </x:c>
+      <x:c r="O29" s="26" t="str">
+        <x:v>9952091294a9603ee53863fca2b454e6a11eb666</x:v>
+      </x:c>
+      <x:c r="P29" s="26" t="str">
+        <x:v>SPARK-197-Newman-Sanitized-Result.json; Admin nonexistent ID</x:v>
+      </x:c>
+      <x:c r="Q29" s="26" t="str">
+        <x:v>API / negative 404</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="50" customHeight="1">
+      <x:c r="B30" s="26" t="str">
+        <x:v>[SP197-GAP-01]</x:v>
+      </x:c>
+      <x:c r="C30" s="26" t="str">
+        <x:v>Duplicate approval via live API</x:v>
+      </x:c>
+      <x:c r="D30" s="26" t="str">
+        <x:v>Replay approve request on already-approved QA application with authorized Admin</x:v>
+      </x:c>
+      <x:c r="E30" s="26" t="str">
+        <x:v>Defined idempotent result; no second provisioning/email</x:v>
+      </x:c>
+      <x:c r="F30" s="26" t="str">
+        <x:v>Dedicated isolated fixture + approval operation IDs</x:v>
+      </x:c>
+      <x:c r="G30" s="72" t="str">
+        <x:v>Untested</x:v>
+      </x:c>
+      <x:c r="H30" s="26"/>
+      <x:c r="I30" s="26"/>
+      <x:c r="J30" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K30" s="26" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L30" s="51" t="n">
+        <x:f>IFERROR(K30/J30,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M30" s="26" t="str">
+        <x:v>Unit duplicate/replay assertions reviewed; not run live</x:v>
+      </x:c>
+      <x:c r="N30" s="26" t="str">
+        <x:v>SPARK-197</x:v>
+      </x:c>
+      <x:c r="O30" s="26" t="str">
+        <x:v>9952091294a9603ee53863fca2b454e6a11eb666</x:v>
+      </x:c>
+      <x:c r="P30" s="26" t="str">
+        <x:v>Jira SPARK-197; OwnerRegistrationService.cs; developer test review</x:v>
+      </x:c>
+      <x:c r="Q30" s="26" t="str">
+        <x:v>TEST / duplicate approval</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="50" customHeight="1">
+      <x:c r="B31" s="26" t="str">
+        <x:v>[SP197-GAP-02]</x:v>
+      </x:c>
+      <x:c r="C31" s="26" t="str">
+        <x:v>Two Admins concurrent approval</x:v>
+      </x:c>
+      <x:c r="D31" s="26" t="str">
+        <x:v>Concurrent POST/PATCH review on same new QA pending application</x:v>
+      </x:c>
+      <x:c r="E31" s="26" t="str">
+        <x:v>Exactly one effective decision; audit and remote side effect consistent</x:v>
+      </x:c>
+      <x:c r="F31" s="26" t="str">
+        <x:v>Two independent authorized Admin sessions and dedicated fixture</x:v>
+      </x:c>
+      <x:c r="G31" s="72" t="str">
+        <x:v>Untested</x:v>
+      </x:c>
+      <x:c r="H31" s="26"/>
+      <x:c r="I31" s="26"/>
+      <x:c r="J31" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K31" s="26" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L31" s="51" t="n">
+        <x:f>IFERROR(K31/J31,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M31" s="26" t="str">
+        <x:v>Prior integration/coordination coverage noted; no real two-Admin HTTP concurrency evidence</x:v>
+      </x:c>
+      <x:c r="N31" s="26" t="str">
+        <x:v>SPARK-197</x:v>
+      </x:c>
+      <x:c r="O31" s="26" t="str">
+        <x:v>9952091294a9603ee53863fca2b454e6a11eb666</x:v>
+      </x:c>
+      <x:c r="P31" s="26" t="str">
+        <x:v>Jira SPARK-197; OwnerRegistrationService.cs; developer test review</x:v>
+      </x:c>
+      <x:c r="Q31" s="26" t="str">
+        <x:v>TEST / concurrency</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="50" customHeight="1">
+      <x:c r="B32" s="26" t="str">
+        <x:v>[SP197-GAP-03]</x:v>
+      </x:c>
+      <x:c r="C32" s="26" t="str">
+        <x:v>Permission revocation of active Admin JWT</x:v>
+      </x:c>
+      <x:c r="D32" s="26" t="str">
+        <x:v>Issue valid token; revoke ACCOUNT_ADMIN/active Admin then call review</x:v>
+      </x:c>
+      <x:c r="E32" s="26" t="str">
+        <x:v>Review blocked after revocation; no unauthorized decision</x:v>
+      </x:c>
+      <x:c r="F32" s="26" t="str">
+        <x:v>Approved isolated security fixture</x:v>
+      </x:c>
+      <x:c r="G32" s="72" t="str">
+        <x:v>Untested</x:v>
+      </x:c>
+      <x:c r="H32" s="26"/>
+      <x:c r="I32" s="26"/>
+      <x:c r="J32" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K32" s="26" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L32" s="51" t="n">
+        <x:f>IFERROR(K32/J32,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M32" s="26" t="str">
+        <x:v>Developer unit test RevokedAdminCannotReadCompletedReplay reviewed; live JWT revoke not run</x:v>
+      </x:c>
+      <x:c r="N32" s="26" t="str">
+        <x:v>SPARK-197</x:v>
+      </x:c>
+      <x:c r="O32" s="26" t="str">
+        <x:v>9952091294a9603ee53863fca2b454e6a11eb666</x:v>
+      </x:c>
+      <x:c r="P32" s="26" t="str">
+        <x:v>Jira SPARK-197; OwnerRegistrationService.cs; developer test review</x:v>
+      </x:c>
+      <x:c r="Q32" s="26" t="str">
+        <x:v>TEST / security</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="50" customHeight="1">
+      <x:c r="B33" s="26" t="str">
+        <x:v>[SP197-GAP-04]</x:v>
+      </x:c>
+      <x:c r="C33" s="26" t="str">
+        <x:v>Approve versus lock/disable race</x:v>
+      </x:c>
+      <x:c r="D33" s="26" t="str">
+        <x:v>Attempt approval concurrently with account disable/lock</x:v>
+      </x:c>
+      <x:c r="E33" s="26" t="str">
+        <x:v>Approval must not unlock separately disabled account</x:v>
+      </x:c>
+      <x:c r="F33" s="26" t="str">
+        <x:v>Approved isolated fixture; role/lock API contract</x:v>
+      </x:c>
+      <x:c r="G33" s="72" t="str">
+        <x:v>Untested</x:v>
+      </x:c>
+      <x:c r="H33" s="26"/>
+      <x:c r="I33" s="26"/>
+      <x:c r="J33" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K33" s="26" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L33" s="51" t="n">
+        <x:f>IFERROR(K33/J33,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M33" s="26" t="str">
+        <x:v>Not performed; cannot infer from active-owner sign-in</x:v>
+      </x:c>
+      <x:c r="N33" s="26" t="str">
+        <x:v>SPARK-197</x:v>
+      </x:c>
+      <x:c r="O33" s="26" t="str">
+        <x:v>9952091294a9603ee53863fca2b454e6a11eb666</x:v>
+      </x:c>
+      <x:c r="P33" s="26" t="str">
+        <x:v>Jira SPARK-197; OwnerRegistrationService.cs; developer test review</x:v>
+      </x:c>
+      <x:c r="Q33" s="26" t="str">
+        <x:v>TEST / state race</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="50" customHeight="1">
+      <x:c r="B34" s="26" t="str">
+        <x:v>[SP197-GAP-05]</x:v>
+      </x:c>
+      <x:c r="C34" s="26" t="str">
+        <x:v>Unverified or missing lot/setup eligibility</x:v>
+      </x:c>
+      <x:c r="D34" s="26" t="str">
+        <x:v>Try approve synthetic pending Owner lacking verification or required lot</x:v>
+      </x:c>
+      <x:c r="E34" s="26" t="str">
+        <x:v>Contract-defined 409/validation failure; no activation</x:v>
+      </x:c>
+      <x:c r="F34" s="26" t="str">
+        <x:v>Isolated incomplete registration fixture</x:v>
+      </x:c>
+      <x:c r="G34" s="72" t="str">
+        <x:v>Untested</x:v>
+      </x:c>
+      <x:c r="H34" s="26"/>
+      <x:c r="I34" s="26"/>
+      <x:c r="J34" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K34" s="26" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L34" s="51" t="n">
+        <x:f>IFERROR(K34/J34,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M34" s="26" t="str">
+        <x:v>Code shows CONTACT_UNVERIFIED/LOT_SETUP_REQUIRED branches; no current live API result</x:v>
+      </x:c>
+      <x:c r="N34" s="26" t="str">
+        <x:v>SPARK-197</x:v>
+      </x:c>
+      <x:c r="O34" s="26" t="str">
+        <x:v>9952091294a9603ee53863fca2b454e6a11eb666</x:v>
+      </x:c>
+      <x:c r="P34" s="26" t="str">
+        <x:v>Jira SPARK-197; OwnerRegistrationService.cs; developer test review</x:v>
+      </x:c>
+      <x:c r="Q34" s="26" t="str">
+        <x:v>TEST / eligibility</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="50" customHeight="1">
+      <x:c r="B35" s="26" t="str">
+        <x:v>[SP197-GAP-06]</x:v>
+      </x:c>
+      <x:c r="C35" s="26" t="str">
+        <x:v>Notification outage after decision</x:v>
+      </x:c>
+      <x:c r="D35" s="26" t="str">
+        <x:v>Force QA-only email delivery failure after approved decision</x:v>
+      </x:c>
+      <x:c r="E35" s="26" t="str">
+        <x:v>Approval persists; delivery separately reports pending/fail and retry</x:v>
+      </x:c>
+      <x:c r="F35" s="26" t="str">
+        <x:v>Controlled QA-only fault injection, not real mailbox</x:v>
+      </x:c>
+      <x:c r="G35" s="72" t="str">
+        <x:v>Untested</x:v>
+      </x:c>
+      <x:c r="H35" s="26"/>
+      <x:c r="I35" s="26"/>
+      <x:c r="J35" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K35" s="26" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L35" s="51" t="n">
+        <x:f>IFERROR(K35/J35,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M35" s="26" t="str">
+        <x:v>Prior PostgreSQL integration test reported; not injected into live QA</x:v>
+      </x:c>
+      <x:c r="N35" s="26" t="str">
+        <x:v>SPARK-197</x:v>
+      </x:c>
+      <x:c r="O35" s="26" t="str">
+        <x:v>9952091294a9603ee53863fca2b454e6a11eb666</x:v>
+      </x:c>
+      <x:c r="P35" s="26" t="str">
+        <x:v>Jira SPARK-197; OwnerRegistrationService.cs; developer test review</x:v>
+      </x:c>
+      <x:c r="Q35" s="26" t="str">
+        <x:v>TEST / dependency failure</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="50" customHeight="1">
+      <x:c r="B36" s="26" t="str">
+        <x:v>[SP197-GAP-07]</x:v>
+      </x:c>
+      <x:c r="C36" s="26" t="str">
+        <x:v>Remote timeout / retry via live API</x:v>
+      </x:c>
+      <x:c r="D36" s="26" t="str">
+        <x:v>Simulate FacilityService failure/timeout; retry approval</x:v>
+      </x:c>
+      <x:c r="E36" s="26" t="str">
+        <x:v>Durable intent; no duplicate site, final decision once</x:v>
+      </x:c>
+      <x:c r="F36" s="26" t="str">
+        <x:v>Dedicated pending QA record and controllable dependency</x:v>
+      </x:c>
+      <x:c r="G36" s="72" t="str">
+        <x:v>Untested</x:v>
+      </x:c>
+      <x:c r="H36" s="26"/>
+      <x:c r="I36" s="26"/>
+      <x:c r="J36" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K36" s="26" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L36" s="51" t="n">
+        <x:f>IFERROR(K36/J36,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M36" s="26" t="str">
+        <x:v>Developer unit assertions reviewed (remote response/local finalize); live HTTP not executed</x:v>
+      </x:c>
+      <x:c r="N36" s="26" t="str">
+        <x:v>SPARK-197</x:v>
+      </x:c>
+      <x:c r="O36" s="26" t="str">
+        <x:v>9952091294a9603ee53863fca2b454e6a11eb666</x:v>
+      </x:c>
+      <x:c r="P36" s="26" t="str">
+        <x:v>Jira SPARK-197; OwnerRegistrationService.cs; developer test review</x:v>
+      </x:c>
+      <x:c r="Q36" s="26" t="str">
+        <x:v>TEST / retry</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="50" customHeight="1">
+      <x:c r="B37" s="26" t="str">
+        <x:v>[SP197-GAP-08]</x:v>
+      </x:c>
+      <x:c r="C37" s="26" t="str">
+        <x:v>Immutable decision audit history</x:v>
+      </x:c>
+      <x:c r="D37" s="26" t="str">
+        <x:v>Inspect audit log entries across transitions and attempted replays</x:v>
+      </x:c>
+      <x:c r="E37" s="26" t="str">
+        <x:v>Traceable actor/time/decision history not overwritten by later attempts</x:v>
+      </x:c>
+      <x:c r="F37" s="26" t="str">
+        <x:v>Audit table/API defined and authorized read access</x:v>
+      </x:c>
+      <x:c r="G37" s="72" t="str">
+        <x:v>Untested</x:v>
+      </x:c>
+      <x:c r="H37" s="26"/>
+      <x:c r="I37" s="26"/>
+      <x:c r="J37" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K37" s="26" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L37" s="51" t="n">
+        <x:f>IFERROR(K37/J37,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M37" s="26" t="str">
+        <x:v>reviewedBy/reviewedAt present; immutable historical log not independently proven</x:v>
+      </x:c>
+      <x:c r="N37" s="26" t="str">
+        <x:v>SPARK-197</x:v>
+      </x:c>
+      <x:c r="O37" s="26" t="str">
+        <x:v>9952091294a9603ee53863fca2b454e6a11eb666</x:v>
+      </x:c>
+      <x:c r="P37" s="26" t="str">
+        <x:v>Jira SPARK-197; OwnerRegistrationService.cs; developer test review</x:v>
+      </x:c>
+      <x:c r="Q37" s="26" t="str">
+        <x:v>TEST / audit history</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="50" customHeight="1">
+      <x:c r="B38" s="26" t="str">
+        <x:v>[SP197-GAP-09]</x:v>
+      </x:c>
+      <x:c r="C38" s="26" t="str">
+        <x:v>Reject/resubmit business rules</x:v>
+      </x:c>
+      <x:c r="D38" s="26" t="str">
+        <x:v>Confirm reject resubmission/appeal behavior with approved SRS decision</x:v>
+      </x:c>
+      <x:c r="E38" s="26" t="str">
+        <x:v>Specified transition/reapply outcome; no invented criteria</x:v>
+      </x:c>
+      <x:c r="F38" s="26" t="str">
+        <x:v>Product/BA decision about reject/resubmit</x:v>
+      </x:c>
+      <x:c r="G38" s="72" t="str">
+        <x:v>Untested</x:v>
+      </x:c>
+      <x:c r="H38" s="26"/>
+      <x:c r="I38" s="26"/>
+      <x:c r="J38" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K38" s="26" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L38" s="51" t="n">
+        <x:f>IFERROR(K38/J38,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M38" s="26" t="str">
+        <x:v>Jira marks detailed reject/resubmit extension unresolved; no independent contract</x:v>
+      </x:c>
+      <x:c r="N38" s="26" t="str">
+        <x:v>SPARK-197</x:v>
+      </x:c>
+      <x:c r="O38" s="26" t="str">
+        <x:v>9952091294a9603ee53863fca2b454e6a11eb666</x:v>
+      </x:c>
+      <x:c r="P38" s="26" t="str">
+        <x:v>Jira SPARK-197; OwnerRegistrationService.cs; developer test review</x:v>
+      </x:c>
+      <x:c r="Q38" s="26" t="str">
+        <x:v>TEST / requirement clarification</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="B1:Q1"/>
+    <x:mergeCell ref="B7:Q7"/>
+    <x:mergeCell ref="B8:Q8"/>
+  </x:mergeCells>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="G10:G80">
+      <x:formula1>"Pass,Fail,Untested,Blocked,N/A"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
@@ -729,7 +2548,7 @@
         <x:v>Last updated</x:v>
       </x:c>
       <x:c r="G5" t="str">
-        <x:v>2026-10-28</x:v>
+        <x:v>2026-10-29</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -896,9 +2715,90 @@
         <x:v>0</x:v>
       </x:c>
     </x:row>
+    <x:row r="15" ht="26" customHeight="1">
+      <x:c r="B15" s="74" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C15" s="75" t="str">
+        <x:v>SP197_Admin_Approval</x:v>
+      </x:c>
+      <x:c r="D15" s="75" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="E15" s="75" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F15" s="75" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="G15" s="75" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H15" s="75" t="n">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="I15" s="78" t="n">
+        <x:f>IFERROR(D15/H15,0)</x:f>
+        <x:v>0.6896551724137931</x:v>
+      </x:c>
+      <x:c r="J15" s="75" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="26" customHeight="1">
+      <x:c r="B16" s="76"/>
+      <x:c r="C16" s="77" t="str">
+        <x:v>Cross-baseline total (reference only)</x:v>
+      </x:c>
+      <x:c r="D16" s="77" t="n">
+        <x:f>D14+D15</x:f>
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="E16" s="77" t="n">
+        <x:f>E14+E15</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F16" s="77" t="n">
+        <x:f>F14+F15</x:f>
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="G16" s="77" t="n">
+        <x:f>G14+G15</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H16" s="77" t="n">
+        <x:f>H14+H15</x:f>
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="I16" s="79" t="n">
+        <x:f>IFERROR(D16/H16,0)</x:f>
+        <x:v>0.6065573770491803</x:v>
+      </x:c>
+      <x:c r="J16" s="77" t="n">
+        <x:f>J14+J15</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="B17" t="str">
+        <x:v>SPARK-197 QA coverage</x:v>
+      </x:c>
+      <x:c r="C17" s="32" t="n">
+        <x:f>IFERROR(D15/H15,0)</x:f>
+        <x:v>0.6896551724137931</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="30" customHeight="1">
+      <x:c r="B18" t="str">
+        <x:v>Note</x:v>
+      </x:c>
+      <x:c r="C18" s="26" t="str">
+        <x:v>Cross-baseline total is indicative; prior PR9 and SPARK-177 results are different SHAs and must NOT be treated as current release sign-off.</x:v>
+      </x:c>
+    </x:row>
     <x:row r="22">
       <x:c r="B22" t="str">
-        <x:v>QA execution coverage</x:v>
+        <x:v>Historical coverage (PR9/SP177 only)</x:v>
       </x:c>
       <x:c r="C22" s="32" t="n">
         <x:f>IFERROR((D14+E14)/H14,0)</x:f>
@@ -910,7 +2810,7 @@
         <x:v>Status / sign-off</x:v>
       </x:c>
       <x:c r="C23" t="str">
-        <x:v>PR9 Owner positive E2E/UI targeted PASS on 05e2976d; SPARK-177 planned scenarios NOT EXECUTED. QA overall not signed off.</x:v>
+        <x:v>Old PR9 05e2976d and SP177 scope unchanged; SPARK197 99520912 partial PASS (20 executed, 9 untested). NOT FINAL QA SIGN-OFF.</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -1107,6 +3007,23 @@
       </x:c>
       <x:c r="F11" s="26" t="str">
         <x:v>Approved auth requirements; safe auth fixtures</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="38" customHeight="1">
+      <x:c r="B12" s="26" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C12" s="26" t="str">
+        <x:v>SP197_Admin_Approval</x:v>
+      </x:c>
+      <x:c r="D12" s="26" t="str">
+        <x:v>SP197_Admin_Approval</x:v>
+      </x:c>
+      <x:c r="E12" s="26" t="str">
+        <x:v>20 executed cases (10 UAT + 10 Newman) + 9 scoped planned gaps; baseline 99520912</x:v>
+      </x:c>
+      <x:c r="F12" s="26" t="str">
+        <x:v>Isolated PR9 QA; Owner A/B synthetic; approved Admin; Newman evidence</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3770,6 +5687,86 @@
         <x:v>PR9_QA_Traceability_Final.xlsx TEST_CASES</x:v>
       </x:c>
     </x:row>
+    <x:row r="15" ht="48" customHeight="1">
+      <x:c r="B15" s="26" t="str">
+        <x:v>SP197-UAT-20261029</x:v>
+      </x:c>
+      <x:c r="C15" s="26" t="str">
+        <x:v>9952091294a9 / 2026-10-29</x:v>
+      </x:c>
+      <x:c r="D15" s="26" t="str">
+        <x:v>Live browser Owner+Admin UAT</x:v>
+      </x:c>
+      <x:c r="E15" s="26" t="str">
+        <x:v>10 distinct PASS manual journey cases</x:v>
+      </x:c>
+      <x:c r="F15" s="26" t="str">
+        <x:v>Real email decision evidence and approved/rejected login. Not full AC sign-off.</x:v>
+      </x:c>
+      <x:c r="G15" s="26" t="str">
+        <x:v>This conversation UAT screenshots; SPARK-197 QA report</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="48" customHeight="1">
+      <x:c r="B16" s="26" t="str">
+        <x:v>SP197-NEW-20261029</x:v>
+      </x:c>
+      <x:c r="C16" s="26" t="str">
+        <x:v>9952091294a9 / 2026-10-29</x:v>
+      </x:c>
+      <x:c r="D16" s="26" t="str">
+        <x:v>Newman API auth and audit</x:v>
+      </x:c>
+      <x:c r="E16" s="26" t="str">
+        <x:v>10 requests / 17 assertions PASS</x:v>
+      </x:c>
+      <x:c r="F16" s="26" t="str">
+        <x:v>Read-only status/authorization with zero-GUID PATCH; no real approval mutation</x:v>
+      </x:c>
+      <x:c r="G16" s="26" t="str">
+        <x:v>SPARK-197-Newman-Sanitized-Result.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="48" customHeight="1">
+      <x:c r="B17" s="26" t="str">
+        <x:v>SP197-UNIT-20261029</x:v>
+      </x:c>
+      <x:c r="C17" s="26" t="str">
+        <x:v>9952091294a9 / 2026-10-29</x:v>
+      </x:c>
+      <x:c r="D17" s="26" t="str">
+        <x:v>Targeted .NET unit run (earlier logs)</x:v>
+      </x:c>
+      <x:c r="E17" s="26" t="str">
+        <x:v>5 pass / 0 fail / 0 skip</x:v>
+      </x:c>
+      <x:c r="F17" s="26" t="str">
+        <x:v>Developer assertion review completed; execution is prior conversation evidence</x:v>
+      </x:c>
+      <x:c r="G17" s="26" t="str">
+        <x:v>OwnerApprovalCoordinationTests.cs; earlier local terminal logs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="48" customHeight="1">
+      <x:c r="B18" s="26" t="str">
+        <x:v>SP197-INTEG-20261029</x:v>
+      </x:c>
+      <x:c r="C18" s="26" t="str">
+        <x:v>9952091294a9 / 2026-10-29</x:v>
+      </x:c>
+      <x:c r="D18" s="26" t="str">
+        <x:v>PostgreSQL integration run (earlier logs)</x:v>
+      </x:c>
+      <x:c r="E18" s="26" t="str">
+        <x:v>5 pass / 0 fail / 0 skip</x:v>
+      </x:c>
+      <x:c r="F18" s="26" t="str">
+        <x:v>No attached raw trx; prior local run log, not Newman</x:v>
+      </x:c>
+      <x:c r="G18" s="26" t="str">
+        <x:v>Earlier local terminal logs; SPARK-197 QA report</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="B1:G1"/>
@@ -4040,6 +6037,106 @@
         <x:v>PR9_QA_Traceability_Final.xlsx</x:v>
       </x:c>
     </x:row>
+    <x:row r="16" ht="52" customHeight="1">
+      <x:c r="B16" s="82" t="str">
+        <x:v>SPARK-197 ENV-COMMIT</x:v>
+      </x:c>
+      <x:c r="C16" s="82" t="str">
+        <x:v>ENVIRONMENT / RESOLVED</x:v>
+      </x:c>
+      <x:c r="D16" s="82" t="str">
+        <x:v>RETEST PASS</x:v>
+      </x:c>
+      <x:c r="E16" s="82" t="str">
+        <x:v>COMMITMENTS_UNAVAILABLE when ReservationService port 5055 was stopped</x:v>
+      </x:c>
+      <x:c r="F16" s="82" t="str">
+        <x:v>Started isolated QA Operations DB + ReservationService; Retry loaded Structure; do not log as Developer bug</x:v>
+      </x:c>
+      <x:c r="G16" s="82" t="str">
+        <x:v>UAT: image(20261029-103705).png; image(20261029-104903).png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="52" customHeight="1">
+      <x:c r="B17" s="83" t="str">
+        <x:v>SPARK-197 CAPACITY</x:v>
+      </x:c>
+      <x:c r="C17" s="83" t="str">
+        <x:v>CONTRACT CLARIFICATION</x:v>
+      </x:c>
+      <x:c r="D17" s="83" t="str">
+        <x:v>NOT CONFIRMED BUG</x:v>
+      </x:c>
+      <x:c r="E17" s="83" t="str">
+        <x:v>10 declared onboarding slots vs physical capacity 0; Structure says no backend slots configured</x:v>
+      </x:c>
+      <x:c r="F17" s="83" t="str">
+        <x:v>Confirm whether approval must instantiate physical slots; avoid importing template count as physical capacity</x:v>
+      </x:c>
+      <x:c r="G17" s="83" t="str">
+        <x:v>UAT: image(20261029-103429).png; image(20261029-104903).png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="52" customHeight="1">
+      <x:c r="B18" s="83" t="str">
+        <x:v>SPARK-197 LIVE-CONC</x:v>
+      </x:c>
+      <x:c r="C18" s="83" t="str">
+        <x:v>TEST GAP</x:v>
+      </x:c>
+      <x:c r="D18" s="83" t="str">
+        <x:v>UNTESTED</x:v>
+      </x:c>
+      <x:c r="E18" s="83" t="str">
+        <x:v>Real two-Admin concurrent decisions and approval-vs-disable race not executed</x:v>
+      </x:c>
+      <x:c r="F18" s="83" t="str">
+        <x:v>Run only with approved isolated pending QA fixtures; unit assertions not live API proof</x:v>
+      </x:c>
+      <x:c r="G18" s="83" t="str">
+        <x:v>Jira SPARK-197 AC; OwnerApprovalCoordinationTests.cs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="52" customHeight="1">
+      <x:c r="B19" s="83" t="str">
+        <x:v>SPARK-197 DELIVERY-FAIL</x:v>
+      </x:c>
+      <x:c r="C19" s="83" t="str">
+        <x:v>TEST GAP</x:v>
+      </x:c>
+      <x:c r="D19" s="83" t="str">
+        <x:v>UNTESTED LIVE</x:v>
+      </x:c>
+      <x:c r="E19" s="83" t="str">
+        <x:v>Real mailbox delivery succeeded; controlled notification outage was not injected</x:v>
+      </x:c>
+      <x:c r="F19" s="83" t="str">
+        <x:v>Review previous PostgreSQL integration evidence; targeted outage requires approved fixture</x:v>
+      </x:c>
+      <x:c r="G19" s="83" t="str">
+        <x:v>OwnerDecision delivery UAT; Jira SPARK-197</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="52" customHeight="1">
+      <x:c r="B20" s="83" t="str">
+        <x:v>SPARK-197 AUDIT</x:v>
+      </x:c>
+      <x:c r="C20" s="83" t="str">
+        <x:v>TEST GAP</x:v>
+      </x:c>
+      <x:c r="D20" s="83" t="str">
+        <x:v>PARTIAL</x:v>
+      </x:c>
+      <x:c r="E20" s="83" t="str">
+        <x:v>Reviewer ID/time present for A/B; immutable historical audit entries not verified</x:v>
+      </x:c>
+      <x:c r="F20" s="83" t="str">
+        <x:v>Confirm audit log/history and permission revocation independently</x:v>
+      </x:c>
+      <x:c r="G20" s="83" t="str">
+        <x:v>SPARK-197 Newman 17/17 + Admin GET detail</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="B1:G1"/>

</xml_diff>